<commit_message>
Backup QR Scanner data - 2026-03-03T11:31:28.641Z - Cache Bust: 1772537488641
</commit_message>
<xml_diff>
--- a/log_history/Y1_B2526_Pharmacology_scanner1772532321064_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
+++ b/log_history/Y1_B2526_Pharmacology_scanner1772532321064_4791e799a156631a1e6528d73ff0b32fbeeb62851b63d680bacede618e9287f5.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Session" sheetId="1" r:id="rId1"/>
+    <sheet name="Scanner" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F73"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -739,9 +739,1129 @@
         <v>marian.samir@med.asu.edu.eg</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>254787</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C18" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D18" t="str">
+        <v>13:25:20</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F18" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>254718</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C19" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D19" t="str">
+        <v>13:25:29</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F19" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>254453</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C20" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D20" t="str">
+        <v>13:25:33</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F20" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>254454</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C21" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D21" t="str">
+        <v>13:25:36</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F21" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>254591</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C22" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D22" t="str">
+        <v>13:25:40</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F22" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>254456</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C23" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D23" t="str">
+        <v>13:25:43</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F23" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>244541</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C24" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D24" t="str">
+        <v>13:25:46</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F24" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>254455</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C25" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D25" t="str">
+        <v>13:25:49</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F25" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>254865</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C26" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D26" t="str">
+        <v>13:25:53</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F26" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>254578</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C27" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D27" t="str">
+        <v>13:25:58</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F27" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>244815</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C28" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D28" t="str">
+        <v>13:26:02</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F28" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>254452</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C29" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D29" t="str">
+        <v>13:26:05</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F29" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>254349</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C30" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D30" t="str">
+        <v>13:26:10</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F30" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>254759</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C31" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D31" t="str">
+        <v>13:26:17</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F31" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>254401</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C32" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D32" t="str">
+        <v>13:26:21</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F32" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>254153</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C33" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D33" t="str">
+        <v>13:26:28</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F33" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>244468</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C34" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D34" t="str">
+        <v>13:26:31</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F34" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>244491</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C35" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D35" t="str">
+        <v>13:26:35</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F35" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>254625</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C36" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D36" t="str">
+        <v>13:26:39</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F36" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>254151</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C37" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D37" t="str">
+        <v>13:26:42</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F37" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>254480</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C38" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D38" t="str">
+        <v>13:26:45</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F38" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>254592</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C39" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D39" t="str">
+        <v>13:26:49</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F39" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>244888</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C40" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D40" t="str">
+        <v>13:26:51</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F40" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>254557</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C41" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D41" t="str">
+        <v>13:26:54</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F41" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>254589</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C42" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D42" t="str">
+        <v>13:26:57</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F42" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>254740</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C43" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D43" t="str">
+        <v>13:27:01</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F43" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>254727</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C44" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D44" t="str">
+        <v>13:27:03</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F44" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>244918</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C45" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D45" t="str">
+        <v>13:27:06</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F45" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>254614</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C46" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D46" t="str">
+        <v>13:27:14</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F46" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>254590</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C47" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D47" t="str">
+        <v>13:27:18</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F47" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>254279</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C48" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D48" t="str">
+        <v>13:27:21</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F48" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>254450</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C49" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D49" t="str">
+        <v>13:27:25</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F49" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>254872</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C50" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D50" t="str">
+        <v>13:27:40</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F50" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>254119</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C51" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D51" t="str">
+        <v>13:27:44</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F51" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>254653</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C52" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D52" t="str">
+        <v>13:27:49</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F52" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>254374</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C53" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D53" t="str">
+        <v>13:27:54</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F53" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>254855</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C54" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D54" t="str">
+        <v>13:27:57</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F54" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>254833</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C55" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D55" t="str">
+        <v>13:28:01</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F55" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>254607</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C56" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D56" t="str">
+        <v>13:28:07</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F56" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>254810</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C57" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D57" t="str">
+        <v>13:28:11</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F57" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>254862</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C58" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D58" t="str">
+        <v>13:28:15</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F58" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>254283</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C59" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D59" t="str">
+        <v>13:28:19</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F59" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>254821</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C60" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D60" t="str">
+        <v>13:28:22</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F60" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>254659</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C61" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D61" t="str">
+        <v>13:28:28</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F61" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>254649</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C62" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D62" t="str">
+        <v>13:28:31</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F62" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="str">
+        <v>254797</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C63" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D63" t="str">
+        <v>13:28:36</v>
+      </c>
+      <c r="E63" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F63" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="str">
+        <v>254875</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C64" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D64" t="str">
+        <v>13:28:41</v>
+      </c>
+      <c r="E64" t="str">
+        <v>Scan</v>
+      </c>
+      <c r="F64" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="str">
+        <v>254411</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C65" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D65" t="str">
+        <v>13:29:04</v>
+      </c>
+      <c r="E65" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F65" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="str">
+        <v>254524</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C66" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D66" t="str">
+        <v>13:29:11</v>
+      </c>
+      <c r="E66" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F66" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="str">
+        <v>254812</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C67" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D67" t="str">
+        <v>13:29:36</v>
+      </c>
+      <c r="E67" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F67" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="str">
+        <v>254458</v>
+      </c>
+      <c r="B68" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C68" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D68" t="str">
+        <v>13:30:32</v>
+      </c>
+      <c r="E68" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F68" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
+        <v>254372</v>
+      </c>
+      <c r="B69" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C69" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D69" t="str">
+        <v>13:30:37</v>
+      </c>
+      <c r="E69" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F69" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>254760</v>
+      </c>
+      <c r="B70" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C70" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D70" t="str">
+        <v>13:30:45</v>
+      </c>
+      <c r="E70" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F70" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="str">
+        <v>254694</v>
+      </c>
+      <c r="B71" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C71" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D71" t="str">
+        <v>13:30:51</v>
+      </c>
+      <c r="E71" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F71" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="str">
+        <v>254565</v>
+      </c>
+      <c r="B72" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C72" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D72" t="str">
+        <v>13:30:59</v>
+      </c>
+      <c r="E72" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F72" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="str">
+        <v>254410</v>
+      </c>
+      <c r="B73" t="str">
+        <v>Pharmacology</v>
+      </c>
+      <c r="C73" t="str">
+        <v>03/03/2026</v>
+      </c>
+      <c r="D73" t="str">
+        <v>13:31:13</v>
+      </c>
+      <c r="E73" t="str">
+        <v>Manual</v>
+      </c>
+      <c r="F73" t="str">
+        <v>marian.samir@med.asu.edu.eg</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F73"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>